<commit_message>
Deliver VD-744 approved B01 gallery and current review evidence
</commit_message>
<xml_diff>
--- a/product generated photo/VD-744/VD-744_LISTING_DRAFT_20261013.xlsx
+++ b/product generated photo/VD-744/VD-744_LISTING_DRAFT_20261013.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Details" sheetId="1" r:id="R1392cf3e4bbf4aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer" sheetId="4" r:id="R5470b915abfb4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety&amp;Compliance" sheetId="5" r:id="R277ee88d7b6441c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Details" sheetId="1" r:id="R699e2b3b29b04dcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer" sheetId="4" r:id="Rb02685f44c374c80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety&amp;Compliance" sheetId="5" r:id="Ra7b701be523c4dc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3710,7 +3710,9 @@
       <x:c r="DG3" s="13" t="str">
         <x:v>GHz</x:v>
       </x:c>
-      <x:c r="DH3" s="13"/>
+      <x:c r="DH3" s="13" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="DI3" s="13" t="n">
         <x:v>256</x:v>
       </x:c>
@@ -3784,13 +3786,27 @@
       <x:c r="ES3" s="13"/>
       <x:c r="ET3" s="13"/>
       <x:c r="EU3" s="13"/>
-      <x:c r="EV3" s="13"/>
-      <x:c r="EW3" s="13"/>
-      <x:c r="EX3" s="13"/>
-      <x:c r="EY3" s="13"/>
-      <x:c r="EZ3" s="13"/>
-      <x:c r="FA3" s="13"/>
-      <x:c r="FB3" s="13"/>
+      <x:c r="EV3" s="13" t="str">
+        <x:v>36 x 182 x 178 mm (horizontal x vertical x front-to-back)</x:v>
+      </x:c>
+      <x:c r="EW3" s="13" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="EX3" s="13" t="str">
+        <x:v>Millimeters</x:v>
+      </x:c>
+      <x:c r="EY3" s="13" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="EZ3" s="13" t="str">
+        <x:v>Millimeters</x:v>
+      </x:c>
+      <x:c r="FA3" s="13" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="FB3" s="13" t="str">
+        <x:v>Millimeters</x:v>
+      </x:c>
       <x:c r="FC3" s="13"/>
       <x:c r="FD3" s="13"/>
       <x:c r="FE3" s="13"/>
@@ -4191,7 +4207,7 @@
         <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="DH4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="DI4" s="19" t="str">
         <x:v>VERIFIED</x:v>
@@ -4311,25 +4327,25 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="EV4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="EW4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="EX4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="EY4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="EZ4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="FA4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="FB4" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="FC4" s="19" t="str">
         <x:v>TBD</x:v>
@@ -4781,7 +4797,7 @@
         <x:v>https://www.intel.com/content/www/us/en/products/sku/241065/intel-core-ultra-7-processor-265t-30m-cache-up-to-5-30-ghz/specifications.html | 2026-10-13 | Exact model/platform evidence; final sold-unit applicability retained separately.</x:v>
       </x:c>
       <x:c r="DH5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | SELLER_INPUT_REQUIRED: select the base sold configuration. Exact ERP child candidates: PD-844 16GB/256GB; PD-850 32GB/512GB; PD-852 16GB/512GB. User confirmed RAM/SSD customization, not a selected baseline or sale tier matrix.</x:v>
+        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/200844 | 2026-10-13 | Exact PD-844 256GB SSD; excludes any external or optional storage.</x:v>
       </x:c>
       <x:c r="DI5" s="17" t="str">
         <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/200844 | 2026-10-13 | Exact PD-844 256GB SSD; excludes any external or optional storage.</x:v>
@@ -4901,25 +4917,25 @@
         <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | SELLER_INPUT_REQUIRED: exact sold-unit SKU/module/label/pack-out evidence required for Keyboard Layout. Series-level options and limits are not installed facts.</x:v>
       </x:c>
       <x:c r="EV5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Upright orientation, as shown in official product views.</x:v>
       </x:c>
       <x:c r="EW5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Upright chassis horizontal width.</x:v>
       </x:c>
       <x:c r="EX5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Exact model/platform evidence; final sold-unit applicability retained separately.</x:v>
       </x:c>
       <x:c r="EY5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Chassis depth.</x:v>
       </x:c>
       <x:c r="EZ5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Exact model/platform evidence; final sold-unit applicability retained separately.</x:v>
       </x:c>
       <x:c r="FA5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Upright chassis vertical height.</x:v>
       </x:c>
       <x:c r="FB5" s="17" t="str">
-        <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | TBD: Dell reports chassis 182mm high x 36mm wide x 178mm deep. Confirm mapping of laptop-oriented template horizontal/vertical/thickness definitions to this desktop before numeric export.</x:v>
+        <x:v>https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | Exact model/platform evidence; final sold-unit applicability retained separately.</x:v>
       </x:c>
       <x:c r="FC5" s="17" t="str">
         <x:v>https://erp-git-feat-part-serial-numbers-overhaul-jtechdigital.vercel.app/products/20744; https://www.dell.com/en-us/shop/desktops/spd/dellpromicroqcm1250 | 2026-10-13 | SELLER_INPUT_REQUIRED: seller/account/fulfillment or compliance owner must supply Software Update Supported to Date for the selected configuration and marketplace; not inferred from OEM options.</x:v>

</xml_diff>